<commit_message>
Add flow diagram, watchdog task comments, and comparator graphs with images
</commit_message>
<xml_diff>
--- a/Investigations/Investigation.xlsx
+++ b/Investigations/Investigation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conor\Documents\College\Masters\Thesis\GeecPE2526\Investigations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Masters\Project\Investigations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2205180-FDFF-4D10-905F-B53FC751CB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2B213A0-2F9F-4800-AA9C-2067E06547C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Consumption" sheetId="1" r:id="rId1"/>
@@ -195,12 +195,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1801,16 +1800,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>34964</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>120569</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>119362</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>60284</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>578733</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>24114</xdr:rowOff>
+      <xdr:colOff>48226</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>156739</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2883,19 +2882,19 @@
         <v>20000</v>
       </c>
       <c r="I10" s="1">
-        <f>$B$1*$B$2*$H10*($B$14+B$15)/$B$3</f>
+        <f t="shared" ref="I10:L12" si="17">$B$1*$B$2*$H10*($B$14+B$15)/$B$3</f>
         <v>8.6800000000000002E-2</v>
       </c>
       <c r="J10" s="1">
-        <f>$B$1*$B$2*$H10*($B$14+C$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>8.9599999999999999E-2</v>
       </c>
       <c r="K10" s="1">
-        <f>$B$1*$B$2*$H10*($B$14+D$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>0.14224000000000001</v>
       </c>
       <c r="L10" s="1">
-        <f>$B$1*$B$2*$H10*($B$14+E$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>4.9279999999999997E-2</v>
       </c>
       <c r="M10" s="2">
@@ -2983,23 +2982,23 @@
       <c r="E11" s="1">
         <v>1.7E-8</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11">
         <v>25000</v>
       </c>
       <c r="I11" s="1">
-        <f>$B$1*$B$2*$H11*($B$14+B$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>0.1085</v>
       </c>
       <c r="J11" s="1">
-        <f>$B$1*$B$2*$H11*($B$14+C$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>0.112</v>
       </c>
       <c r="K11" s="1">
-        <f>$B$1*$B$2*$H11*($B$14+D$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>0.17780000000000001</v>
       </c>
       <c r="L11" s="1">
-        <f>$B$1*$B$2*$H11*($B$14+E$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>6.1599999999999995E-2</v>
       </c>
       <c r="M11" s="2">
@@ -3091,19 +3090,19 @@
         <v>30000</v>
       </c>
       <c r="I12" s="1">
-        <f>$B$1*$B$2*$H12*($B$14+B$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>0.13020000000000001</v>
       </c>
       <c r="J12" s="1">
-        <f>$B$1*$B$2*$H12*($B$14+C$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>0.13440000000000002</v>
       </c>
       <c r="K12" s="1">
-        <f>$B$1*$B$2*$H12*($B$14+D$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>0.21336000000000002</v>
       </c>
       <c r="L12" s="1">
-        <f>$B$1*$B$2*$H12*($B$14+E$15)/$B$3</f>
+        <f t="shared" si="17"/>
         <v>7.392E-2</v>
       </c>
       <c r="M12" s="2">
@@ -3240,7 +3239,7 @@
         <v>4.0999999999999997E-8</v>
       </c>
       <c r="C17" s="1">
-        <f t="shared" ref="C17:E17" si="17">$B$6+0.0000000093</f>
+        <f t="shared" ref="C17" si="18">$B$6+0.0000000093</f>
         <v>1.9300000000000001E-8</v>
       </c>
       <c r="D17" s="1">
@@ -3261,7 +3260,7 @@
         <v>3.55E-8</v>
       </c>
       <c r="C18" s="1">
-        <f t="shared" ref="C18:E18" si="18">$B$6+0.0000000061</f>
+        <f t="shared" ref="C18" si="19">$B$6+0.0000000061</f>
         <v>1.6099999999999999E-8</v>
       </c>
       <c r="D18" s="1">

</xml_diff>